<commit_message>
Comprehensive import template: all discipline spec fields
Template now includes every engineering input from the Parameter Dictionary grouped/colour-coded by discipline (Electrical, Water/Plumbing, Drainage, Gas, Ventilation) plus Dimensions & Clearances. Fill applicable, leave rest blank.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/EOS_Import_Template.xlsx
+++ b/EOS_Import_Template.xlsx
@@ -93,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="266">
   <si>
     <t>Equipment Family *</t>
   </si>
@@ -128,28 +128,79 @@
     <t>Product Image</t>
   </si>
   <si>
+    <t>Phase</t>
+  </si>
+  <si>
     <t>Voltage (V)</t>
   </si>
   <si>
-    <t>Phase</t>
-  </si>
-  <si>
-    <t>Total Power (kW)</t>
+    <t>Frequency (Hz)</t>
+  </si>
+  <si>
+    <t>Power (kW)</t>
   </si>
   <si>
     <t>Current (A)</t>
   </si>
   <si>
-    <t>Width (mm)</t>
-  </si>
-  <si>
-    <t>Depth (mm)</t>
-  </si>
-  <si>
-    <t>Height (mm)</t>
-  </si>
-  <si>
-    <t>Weight (kg)</t>
+    <t>Water Pressure (kPa)</t>
+  </si>
+  <si>
+    <t>Water Inlet Size</t>
+  </si>
+  <si>
+    <t>Water Requirement</t>
+  </si>
+  <si>
+    <t>Water Hardness</t>
+  </si>
+  <si>
+    <t>Drain Size</t>
+  </si>
+  <si>
+    <t>Drain Requirement</t>
+  </si>
+  <si>
+    <t>Drain Type</t>
+  </si>
+  <si>
+    <t>Gas Type</t>
+  </si>
+  <si>
+    <t>Gas Pressure (mbar)</t>
+  </si>
+  <si>
+    <t>Gas Power (kW)</t>
+  </si>
+  <si>
+    <t>Gas Consumption</t>
+  </si>
+  <si>
+    <t>Gas Connection Size</t>
+  </si>
+  <si>
+    <t>Heat Load (kW)</t>
+  </si>
+  <si>
+    <t>Overall Width (mm)</t>
+  </si>
+  <si>
+    <t>Overall Depth (mm)</t>
+  </si>
+  <si>
+    <t>Overall Height (mm)</t>
+  </si>
+  <si>
+    <t>Net Weight (kg)</t>
+  </si>
+  <si>
+    <t>Rear Clearance (mm)</t>
+  </si>
+  <si>
+    <t>Side Clearance (mm)</t>
+  </si>
+  <si>
+    <t>Top Clearance (mm)</t>
   </si>
   <si>
     <t>Cooking</t>
@@ -185,75 +236,81 @@
     <t>3</t>
   </si>
   <si>
+    <t>Gas Range</t>
+  </si>
+  <si>
+    <t>GR-6B-01</t>
+  </si>
+  <si>
+    <t>6-Burner Gas Range</t>
+  </si>
+  <si>
+    <t>MBM</t>
+  </si>
+  <si>
+    <t>Magistra</t>
+  </si>
+  <si>
+    <t>Gas</t>
+  </si>
+  <si>
+    <t>6 open burners</t>
+  </si>
+  <si>
+    <t>NG / LPG</t>
+  </si>
+  <si>
+    <t>Bakery Equipment</t>
+  </si>
+  <si>
+    <t>Beverage Equipment</t>
+  </si>
+  <si>
+    <t>Food Preparation</t>
+  </si>
+  <si>
+    <t>Ice Machines</t>
+  </si>
+  <si>
+    <t>Laundry Equipment</t>
+  </si>
+  <si>
     <t>Refrigeration</t>
   </si>
   <si>
+    <t>Serving &amp; Distribution</t>
+  </si>
+  <si>
+    <t>Stainless Steel Fabrication</t>
+  </si>
+  <si>
+    <t>Ventilation</t>
+  </si>
+  <si>
+    <t>Warewashing</t>
+  </si>
+  <si>
+    <t>Waste Management</t>
+  </si>
+  <si>
+    <t>Dough Divider</t>
+  </si>
+  <si>
+    <t>Espresso Machine</t>
+  </si>
+  <si>
+    <t>Vegetable Cutter</t>
+  </si>
+  <si>
+    <t>Modular Ice Machine</t>
+  </si>
+  <si>
+    <t>Washer Extractor</t>
+  </si>
+  <si>
     <t>Reach-In Refrigerator</t>
   </si>
   <si>
-    <t>REF-EX-01</t>
-  </si>
-  <si>
-    <t>Upright Refrigerator 600L</t>
-  </si>
-  <si>
-    <t>MBM</t>
-  </si>
-  <si>
-    <t>Single-door reach-in</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Bakery Equipment</t>
-  </si>
-  <si>
-    <t>Beverage Equipment</t>
-  </si>
-  <si>
-    <t>Food Preparation</t>
-  </si>
-  <si>
-    <t>Ice Machines</t>
-  </si>
-  <si>
-    <t>Laundry Equipment</t>
-  </si>
-  <si>
-    <t>Serving &amp; Distribution</t>
-  </si>
-  <si>
-    <t>Stainless Steel Fabrication</t>
-  </si>
-  <si>
-    <t>Ventilation</t>
-  </si>
-  <si>
-    <t>Warewashing</t>
-  </si>
-  <si>
-    <t>Waste Management</t>
-  </si>
-  <si>
-    <t>Dough Divider</t>
-  </si>
-  <si>
-    <t>Espresso Machine</t>
-  </si>
-  <si>
-    <t>Gas Range</t>
-  </si>
-  <si>
-    <t>Vegetable Cutter</t>
-  </si>
-  <si>
-    <t>Modular Ice Machine</t>
-  </si>
-  <si>
-    <t>Washer Extractor</t>
-  </si>
-  <si>
     <t>Heated Trolley</t>
   </si>
   <si>
@@ -797,49 +854,43 @@
     <t>HOW TO USE</t>
   </si>
   <si>
-    <t>1.  One row = one product. Fill the 'Products' sheet (the first tab).</t>
+    <t>1.  One row = one product. Fill the 'Products' sheet (the first tab). Fill the columns that apply and LEAVE THE REST BLANK.</t>
   </si>
   <si>
     <t>2.  Columns marked * are REQUIRED: Equipment Family, Equipment Category, Product Code, Product Name, Brand / Manufacturer.</t>
   </si>
   <si>
-    <t>3.  Equipment Family — pick from the dropdown (12 families).</t>
-  </si>
-  <si>
-    <t>4.  Equipment Category — pick from the dropdown; it is filtered by the Family you selected.</t>
-  </si>
-  <si>
-    <t>5.  Product Code — the UNIQUE identifier. EOS uses it to recognise the item on re-import, so keep it stable and never reuse a code.</t>
-  </si>
-  <si>
-    <t>6.  Brand / Manufacturer = the maker (e.g. MBM). Put the product line in 'Series / Line' (e.g. Magistra).</t>
-  </si>
-  <si>
-    <t>7.  Power Type — Electric, Gas or Neutral.</t>
-  </si>
-  <si>
-    <t>8.  Product Image — paste the picture directly INTO the cell (optional). You may also supply images named by code separately.</t>
-  </si>
-  <si>
-    <t>9.  Any EXTRA column you add (e.g. Voltage, Total Power, Gas Pressure) becomes an engineering specification automatically.</t>
-  </si>
-  <si>
-    <t>10. Imported items arrive as DRAFT for review before they are approved.</t>
+    <t>3.  Equipment Family — pick from the dropdown (12 families).  Equipment Category — dropdown filtered by the Family you chose.</t>
+  </si>
+  <si>
+    <t>4.  Product Code — the UNIQUE identifier. EOS uses it to recognise the item on re-import, so keep it stable and never reuse a code.</t>
+  </si>
+  <si>
+    <t>5.  Brand / Manufacturer = the maker (e.g. MBM). Put the product line in 'Series / Line' (e.g. Magistra).</t>
+  </si>
+  <si>
+    <t>6.  Engineering columns are grouped and colour-coded by discipline: Electrical, Water/Plumbing, Drainage, Gas, Ventilation, and Dimensions &amp; Clearances.</t>
+  </si>
+  <si>
+    <t>7.  You can ADD your own extra columns too — any extra header becomes an engineering attribute automatically.</t>
+  </si>
+  <si>
+    <t>8.  EOS computes the 'Recommended …' values (cable size, breaker, pipe size, clearances, airflow…) from these inputs, so those are NOT in the template.</t>
+  </si>
+  <si>
+    <t>9.  Product Image — paste the picture directly INTO the cell (optional). Imported items arrive as DRAFT for review.</t>
   </si>
   <si>
     <t>RE-IMPORT / UPDATES</t>
   </si>
   <si>
-    <t>• EOS matches items by Product Code: existing items are UPDATED (a new draft version), new items are ADDED — you never delete and re-import everything.</t>
-  </si>
-  <si>
-    <t>• Renaming a code creates a NEW item (the old one stays). Keep codes stable.</t>
+    <t>• EOS matches items by Product Code: existing items are UPDATED, new items are ADDED — you never delete and re-import everything. Renaming a code creates a NEW item.</t>
   </si>
   <si>
     <t>REFERENCE</t>
   </si>
   <si>
-    <t>• The 'Families &amp; Categories' sheet lists every valid Family and its Categories (12 families, 194 categories).</t>
+    <t>• 'Families &amp; Categories' sheet — every valid Family and its Categories (12 families, 194 categories).</t>
   </si>
 </sst>
 </file>
@@ -857,6 +908,7 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
     </font>
     <font>
       <b/>
@@ -870,7 +922,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -889,7 +941,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF6B7280"/>
+        <fgColor rgb="FF0E7490"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1D4ED8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0F766E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB91C1C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7C3AED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4D7C0F"/>
       </patternFill>
     </fill>
     <fill>
@@ -910,7 +987,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -921,7 +998,22 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -1263,7 +1355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S600"/>
+  <dimension ref="A1:AJ600"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1273,17 +1365,28 @@
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="8" max="8" width="28" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="10" max="10" width="22" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="12" customWidth="1"/>
-    <col min="13" max="13" width="10" customWidth="1"/>
-    <col min="14" max="14" width="14" customWidth="1"/>
-    <col min="15" max="19" width="12" customWidth="1"/>
+    <col min="12" max="16" width="12" customWidth="1"/>
+    <col min="17" max="17" width="17" customWidth="1"/>
+    <col min="18" max="18" width="19" customWidth="1"/>
+    <col min="19" max="19" width="20" customWidth="1"/>
+    <col min="20" max="20" width="17" customWidth="1"/>
+    <col min="21" max="21" width="13" customWidth="1"/>
+    <col min="22" max="22" width="20" customWidth="1"/>
+    <col min="23" max="23" width="13" customWidth="1"/>
+    <col min="24" max="24" width="12" customWidth="1"/>
+    <col min="25" max="25" width="15" customWidth="1"/>
+    <col min="26" max="26" width="12" customWidth="1"/>
+    <col min="27" max="27" width="18" customWidth="1"/>
+    <col min="28" max="28" width="22" customWidth="1"/>
+    <col min="29" max="29" width="12" customWidth="1"/>
+    <col min="30" max="36" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1332,132 +1435,285 @@
       <c r="P1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="S1" s="4" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="B2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H2" t="s">
+        <v>43</v>
+      </c>
+      <c r="I2" t="s">
+        <v>44</v>
+      </c>
+      <c r="J2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K2" t="s">
+        <v>45</v>
+      </c>
+      <c r="L2" t="s">
+        <v>46</v>
+      </c>
+      <c r="M2">
+        <v>400</v>
+      </c>
+      <c r="N2">
+        <v>50</v>
+      </c>
+      <c r="O2">
+        <v>18.9</v>
+      </c>
+      <c r="P2">
+        <v>32</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>45</v>
+      </c>
+      <c r="R2" t="s">
+        <v>45</v>
+      </c>
+      <c r="S2" t="s">
+        <v>45</v>
+      </c>
+      <c r="T2" t="s">
+        <v>45</v>
+      </c>
+      <c r="U2" t="s">
+        <v>45</v>
+      </c>
+      <c r="V2" t="s">
+        <v>45</v>
+      </c>
+      <c r="W2" t="s">
+        <v>45</v>
+      </c>
+      <c r="X2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AD2">
+        <v>860</v>
+      </c>
+      <c r="AE2">
+        <v>750</v>
+      </c>
+      <c r="AF2">
+        <v>1010</v>
+      </c>
+      <c r="AG2">
+        <v>120</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I3" t="s">
+        <v>44</v>
+      </c>
+      <c r="J3" t="s">
+        <v>45</v>
+      </c>
+      <c r="K3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L3" t="s">
+        <v>45</v>
+      </c>
+      <c r="M3" t="s">
+        <v>45</v>
+      </c>
+      <c r="N3" t="s">
+        <v>45</v>
+      </c>
+      <c r="O3" t="s">
+        <v>45</v>
+      </c>
+      <c r="P3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>45</v>
+      </c>
+      <c r="R3" t="s">
+        <v>45</v>
+      </c>
+      <c r="S3" t="s">
+        <v>45</v>
+      </c>
+      <c r="T3" t="s">
+        <v>45</v>
+      </c>
+      <c r="U3" t="s">
+        <v>45</v>
+      </c>
+      <c r="V3" t="s">
+        <v>45</v>
+      </c>
+      <c r="W3" t="s">
+        <v>45</v>
+      </c>
+      <c r="X3" t="s">
+        <v>54</v>
+      </c>
+      <c r="Y3">
         <v>20</v>
       </c>
-      <c r="C2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F2" t="s">
-        <v>24</v>
-      </c>
-      <c r="G2" t="s">
-        <v>25</v>
-      </c>
-      <c r="H2" t="s">
-        <v>26</v>
-      </c>
-      <c r="I2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K2" t="s">
-        <v>28</v>
-      </c>
-      <c r="L2">
-        <v>400</v>
-      </c>
-      <c r="M2" t="s">
-        <v>29</v>
-      </c>
-      <c r="N2">
-        <v>18.9</v>
-      </c>
-      <c r="O2">
-        <v>32</v>
-      </c>
-      <c r="P2">
-        <v>860</v>
-      </c>
-      <c r="Q2">
-        <v>750</v>
-      </c>
-      <c r="R2">
-        <v>1010</v>
-      </c>
-      <c r="S2">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="Z3">
         <v>33</v>
       </c>
-      <c r="E3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" t="s">
-        <v>35</v>
-      </c>
-      <c r="I3" t="s">
-        <v>27</v>
-      </c>
-      <c r="J3" t="s">
-        <v>28</v>
-      </c>
-      <c r="K3" t="s">
-        <v>28</v>
-      </c>
-      <c r="L3">
-        <v>230</v>
-      </c>
-      <c r="M3" t="s">
-        <v>36</v>
-      </c>
-      <c r="N3">
-        <v>0.3</v>
-      </c>
-      <c r="O3">
-        <v>2</v>
-      </c>
-      <c r="P3">
-        <v>700</v>
-      </c>
-      <c r="Q3">
-        <v>800</v>
-      </c>
-      <c r="R3">
-        <v>2000</v>
-      </c>
-      <c r="S3">
-        <v>110</v>
+      <c r="AA3" t="s">
+        <v>45</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>45</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>45</v>
+      </c>
+      <c r="AD3">
+        <v>900</v>
+      </c>
+      <c r="AE3">
+        <v>900</v>
+      </c>
+      <c r="AF3">
+        <v>850</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>45</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>45</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>45</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25"/>
@@ -3900,685 +4156,685 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>46</v>
+      <c r="A1" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" t="s">
         <v>47</v>
       </c>
-      <c r="B2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C2" t="s">
-        <v>49</v>
-      </c>
       <c r="D2" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="E2" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="F2" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="G2" t="s">
-        <v>31</v>
+        <v>71</v>
       </c>
       <c r="H2" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="I2" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="J2" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="K2" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="L2" t="s">
-        <v>57</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="C3" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="D3" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="E3" t="s">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="F3" t="s">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="G3" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="H3" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="I3" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="J3" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="K3" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="L3" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
+        <v>90</v>
       </c>
       <c r="C4" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="D4" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="E4" t="s">
-        <v>74</v>
+        <v>93</v>
       </c>
       <c r="F4" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="G4" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="H4" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="I4" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="J4" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="K4" t="s">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="L4" t="s">
-        <v>81</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>82</v>
+        <v>101</v>
       </c>
       <c r="B5" t="s">
-        <v>83</v>
+        <v>102</v>
       </c>
       <c r="C5" t="s">
-        <v>84</v>
+        <v>103</v>
       </c>
       <c r="D5" t="s">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="E5" t="s">
-        <v>86</v>
+        <v>105</v>
       </c>
       <c r="F5" t="s">
-        <v>87</v>
+        <v>106</v>
       </c>
       <c r="G5" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="H5" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="I5" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="J5" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="K5" t="s">
-        <v>92</v>
+        <v>111</v>
       </c>
       <c r="L5" t="s">
-        <v>93</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
       <c r="B6" t="s">
-        <v>95</v>
+        <v>114</v>
       </c>
       <c r="C6" t="s">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="D6" t="s">
-        <v>97</v>
+        <v>116</v>
       </c>
       <c r="E6" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="F6" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="G6" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="H6" t="s">
-        <v>101</v>
+        <v>120</v>
       </c>
       <c r="I6" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="J6" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="K6" t="s">
-        <v>104</v>
+        <v>123</v>
       </c>
       <c r="L6" t="s">
-        <v>105</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>106</v>
+        <v>125</v>
       </c>
       <c r="B7" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="C7" t="s">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="D7" t="s">
-        <v>109</v>
+        <v>128</v>
       </c>
       <c r="E7" t="s">
-        <v>110</v>
+        <v>129</v>
       </c>
       <c r="F7" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
       <c r="G7" t="s">
-        <v>112</v>
+        <v>131</v>
       </c>
       <c r="H7" t="s">
-        <v>113</v>
+        <v>132</v>
       </c>
       <c r="I7" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="J7" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="K7" t="s">
-        <v>116</v>
+        <v>135</v>
       </c>
       <c r="L7" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="B8" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="C8" t="s">
-        <v>120</v>
+        <v>139</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="E8" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="F8" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="G8" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
       <c r="H8" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="I8" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
       <c r="J8" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="K8" t="s">
-        <v>127</v>
+        <v>146</v>
       </c>
       <c r="L8" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
       <c r="B9" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
       <c r="C9" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="D9" t="s">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="E9" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="F9" t="s">
-        <v>133</v>
+        <v>152</v>
       </c>
       <c r="G9" t="s">
-        <v>134</v>
+        <v>153</v>
       </c>
       <c r="H9" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="I9" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="J9" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="K9" t="s">
-        <v>138</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>139</v>
+        <v>158</v>
       </c>
       <c r="B10" t="s">
-        <v>140</v>
+        <v>159</v>
       </c>
       <c r="C10" t="s">
-        <v>141</v>
+        <v>160</v>
       </c>
       <c r="D10" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="F10" t="s">
-        <v>142</v>
+        <v>161</v>
       </c>
       <c r="G10" t="s">
-        <v>143</v>
+        <v>162</v>
       </c>
       <c r="H10" t="s">
-        <v>144</v>
+        <v>163</v>
       </c>
       <c r="I10" t="s">
-        <v>145</v>
+        <v>164</v>
       </c>
       <c r="J10" t="s">
-        <v>146</v>
+        <v>165</v>
       </c>
       <c r="K10" t="s">
-        <v>147</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>148</v>
+        <v>167</v>
       </c>
       <c r="B11" t="s">
-        <v>149</v>
+        <v>168</v>
       </c>
       <c r="C11" t="s">
-        <v>150</v>
+        <v>169</v>
       </c>
       <c r="D11" t="s">
-        <v>148</v>
+        <v>167</v>
       </c>
       <c r="F11" t="s">
-        <v>151</v>
+        <v>170</v>
       </c>
       <c r="G11" t="s">
-        <v>152</v>
+        <v>171</v>
       </c>
       <c r="H11" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="I11" t="s">
-        <v>154</v>
+        <v>173</v>
       </c>
       <c r="J11" t="s">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="K11" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="B12" t="s">
-        <v>158</v>
+        <v>177</v>
       </c>
       <c r="C12" t="s">
-        <v>159</v>
+        <v>178</v>
       </c>
       <c r="D12" t="s">
-        <v>160</v>
+        <v>179</v>
       </c>
       <c r="F12" t="s">
-        <v>161</v>
+        <v>180</v>
       </c>
       <c r="G12" t="s">
-        <v>162</v>
+        <v>181</v>
       </c>
       <c r="H12" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
       <c r="I12" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="J12" t="s">
-        <v>165</v>
+        <v>184</v>
       </c>
       <c r="K12" t="s">
-        <v>166</v>
+        <v>185</v>
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>167</v>
+        <v>186</v>
       </c>
       <c r="C13" t="s">
-        <v>168</v>
+        <v>187</v>
       </c>
       <c r="D13" t="s">
-        <v>169</v>
+        <v>188</v>
       </c>
       <c r="G13" t="s">
-        <v>170</v>
+        <v>189</v>
       </c>
       <c r="I13" t="s">
-        <v>171</v>
+        <v>190</v>
       </c>
       <c r="K13" t="s">
-        <v>172</v>
+        <v>191</v>
       </c>
     </row>
     <row r="14" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>173</v>
+        <v>192</v>
       </c>
       <c r="D14" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="G14" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="I14" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
     </row>
     <row r="15" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>177</v>
+        <v>196</v>
       </c>
       <c r="D15" t="s">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="G15" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="I15" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
     </row>
     <row r="16" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C16" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="D16" t="s">
-        <v>182</v>
+        <v>201</v>
       </c>
       <c r="G16" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="I16" t="s">
-        <v>184</v>
+        <v>203</v>
       </c>
     </row>
     <row r="17" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C17" t="s">
-        <v>185</v>
+        <v>204</v>
       </c>
       <c r="D17" t="s">
-        <v>186</v>
+        <v>205</v>
       </c>
       <c r="G17" t="s">
-        <v>187</v>
+        <v>206</v>
       </c>
       <c r="I17" t="s">
-        <v>188</v>
+        <v>207</v>
       </c>
     </row>
     <row r="18" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C18" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="D18" t="s">
-        <v>189</v>
+        <v>208</v>
       </c>
       <c r="G18" t="s">
-        <v>190</v>
+        <v>209</v>
       </c>
       <c r="I18" t="s">
-        <v>191</v>
+        <v>210</v>
       </c>
     </row>
     <row r="19" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
-        <v>192</v>
+        <v>211</v>
       </c>
       <c r="D19" t="s">
-        <v>193</v>
+        <v>212</v>
       </c>
       <c r="G19" t="s">
-        <v>194</v>
+        <v>213</v>
       </c>
       <c r="I19" t="s">
-        <v>195</v>
+        <v>214</v>
       </c>
     </row>
     <row r="20" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
-        <v>139</v>
+        <v>158</v>
       </c>
       <c r="D20" t="s">
-        <v>196</v>
+        <v>215</v>
       </c>
       <c r="G20" t="s">
-        <v>197</v>
+        <v>216</v>
       </c>
       <c r="I20" t="s">
-        <v>198</v>
+        <v>217</v>
       </c>
     </row>
     <row r="21" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C21" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="D21" t="s">
-        <v>200</v>
+        <v>219</v>
       </c>
       <c r="G21" t="s">
-        <v>201</v>
+        <v>220</v>
       </c>
       <c r="I21" t="s">
-        <v>202</v>
+        <v>221</v>
       </c>
     </row>
     <row r="22" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C22" t="s">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="D22" t="s">
-        <v>203</v>
+        <v>222</v>
       </c>
       <c r="G22" t="s">
-        <v>204</v>
+        <v>223</v>
       </c>
       <c r="I22" t="s">
-        <v>205</v>
+        <v>224</v>
       </c>
     </row>
     <row r="23" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C23" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
       <c r="D23" t="s">
-        <v>206</v>
+        <v>225</v>
       </c>
       <c r="G23" t="s">
-        <v>207</v>
+        <v>226</v>
       </c>
       <c r="I23" t="s">
-        <v>208</v>
+        <v>227</v>
       </c>
     </row>
     <row r="24" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C24" t="s">
-        <v>209</v>
+        <v>228</v>
       </c>
       <c r="D24" t="s">
-        <v>210</v>
+        <v>229</v>
       </c>
       <c r="G24" t="s">
-        <v>211</v>
+        <v>230</v>
       </c>
     </row>
     <row r="25" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C25" t="s">
-        <v>212</v>
+        <v>231</v>
       </c>
       <c r="D25" t="s">
-        <v>213</v>
+        <v>232</v>
       </c>
       <c r="G25" t="s">
-        <v>214</v>
+        <v>233</v>
       </c>
     </row>
     <row r="26" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C26" t="s">
-        <v>215</v>
+        <v>234</v>
       </c>
       <c r="D26" t="s">
-        <v>216</v>
+        <v>235</v>
       </c>
       <c r="G26" t="s">
-        <v>217</v>
+        <v>236</v>
       </c>
     </row>
     <row r="27" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C27" t="s">
-        <v>218</v>
+        <v>237</v>
       </c>
       <c r="D27" t="s">
-        <v>219</v>
+        <v>238</v>
       </c>
       <c r="G27" t="s">
-        <v>220</v>
+        <v>239</v>
       </c>
     </row>
     <row r="28" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C28" t="s">
-        <v>221</v>
+        <v>240</v>
       </c>
       <c r="D28" t="s">
-        <v>222</v>
+        <v>241</v>
       </c>
       <c r="G28" t="s">
-        <v>223</v>
+        <v>242</v>
       </c>
     </row>
     <row r="29" spans="3:7" x14ac:dyDescent="0.25">
       <c r="C29" t="s">
-        <v>224</v>
+        <v>243</v>
       </c>
       <c r="D29" t="s">
-        <v>225</v>
+        <v>244</v>
       </c>
       <c r="G29" t="s">
-        <v>226</v>
+        <v>245</v>
       </c>
     </row>
     <row r="30" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C30" t="s">
-        <v>227</v>
+        <v>246</v>
       </c>
       <c r="D30" t="s">
-        <v>228</v>
+        <v>247</v>
       </c>
     </row>
     <row r="31" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C31" t="s">
-        <v>229</v>
+        <v>248</v>
       </c>
       <c r="D31" t="s">
-        <v>230</v>
+        <v>249</v>
       </c>
     </row>
     <row r="32" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C32" t="s">
-        <v>231</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -4589,171 +4845,155 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
-    <col min="2" max="2" width="112" customWidth="1"/>
+    <col min="2" max="2" width="116" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>232</v>
+        <v>45</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>233</v>
+        <v>45</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="B4" t="s">
-        <v>234</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="B5" t="s">
-        <v>235</v>
+        <v>254</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>236</v>
+        <v>255</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>237</v>
+        <v>256</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>238</v>
+        <v>257</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="B9" t="s">
-        <v>239</v>
+        <v>258</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="B10" t="s">
-        <v>240</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="B11" t="s">
-        <v>241</v>
+        <v>260</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="B12" t="s">
-        <v>242</v>
+        <v>261</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="B13" t="s">
-        <v>243</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" t="s">
-        <v>28</v>
+        <v>45</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>244</v>
+        <v>45</v>
+      </c>
+      <c r="B15" t="s">
+        <v>263</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="B16" t="s">
-        <v>245</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" t="s">
-        <v>246</v>
+        <v>45</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="B18" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>28</v>
-      </c>
-      <c r="B20" t="s">
-        <v>248</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>

</xml_diff>